<commit_message>
Versão com Output do Reasoning e Grid - sem validação e votação
Os dados agora são tidos apenas por reasoning e grid, sem a correção de se está certo ou errado. Assim, o jeito será enviar as tasks para o Gemini Pro, junto dos dados da tabela, e pedir para ele fazer uma análise e correção deles.
</commit_message>
<xml_diff>
--- a/batch_results.xlsx
+++ b/batch_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,84 +436,9 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CORRECT
-Reasoning:
-*   Example 1 Input:
-        0 0 0 0 0 0 0
-        0 8 0 0 0 0 0
-        0 8 8 0 0 0 0
-        0 0 0 0 8 8 0
-        0 0 0 0 0 8 0
-        0 0 0 0 0 0 0
-        0 0 0 0 0 0 0
-    *   Example 1 Output:
-        0 0 0 0 0 0 0
-        0 8 1 0 0 0 0
-        0 8 8 0 0 0 0
-        0 0 0 0 8 8 0
-        0 0 0 0 1 8 0
-        0 0 0 0 0 0 0
-        0 0 0 0 0 0 0
-    *   Observation 1: The color 8 forms shapes.
-        Shape 1: (1,1), (2,1), (2,2) - a small L-shape (inverted L).
-        Shape 2: (3,4), (3,5), (4,5) - a small L-shape.
-    *   Observation 2: In the output, some 0s became 1s.
-        (1,2) became 1. (1,2) is the empty space that would complete the 2x2 square containing (1,1), (2,1), (2,2).
-        (4,4) became 1. (4,4) is the empty space that would complete the 2x2 square containing (3,4), (3,5), (4,5).
-    *   Example 2 Input:
-        0 0 0 0 8 8 0
-        0 0 0 0 0 8 0
-        0 0 8 0 0 0 0
-        0 0 8 8 0 0 0
-        0 0 0 0 0 0 0
-        0 0 0 0 8 0 0
-        0 0 0 8 8 0 0
-    *   Example 2 Output:
-        0 0 0 0 8 8 0
-        0 0 0 0 1 8 0
-        0 0 8 1 0 0 0
-        0 0 8 8 0 0 0
-        0 0 0 0 0 0 0
-        0 0 0 1 8 0 0
-        0 0 0 8 8 0 0
-    *   Observation 1: The color 8 forms shapes.
-        Shape 1: (0,4), (0,5), (1,5) - an L-shape.
-        Shape 2: (2,2), (3,2), (3,3) - an L-shape.
-        Shape 3: (5,4), (6,3), (6,4) - an L-shape.
-    *   Observation 2: In the output, some 0s became 1s.
-        (1,4) became 1. (1,4) completes the 2x2 square with (0,4), (0,5), (1,5).
-        (2,3) became 1. (2,3) completes the 2x2 square with (2,2), (3,2), (3,3).
-        (5,3) became 1. (5,3) completes the 2x2 square with (5,4), (6,3), (6,4).
-    *   The rule seems to be: Identify all 3-pixel L-shaped figures formed by the color 8.
-    *   Each 3-pixel L-shape fits within a 2x2 square.
-    *   Fill the remaining empty cell (the 4th cell) of that 2x2 square with the color 1.
-    *   Test Input:
-        0 0 0 0 0 8 8 (Row 0)
-        8 8 0 0 0 0 8 (Row 1)
-        8 0 0 0 0 0 0 (Row 2)
-        0 0 0 8 0 0 0 (Row 3)
-        0 0 0 8 8 0 0 (Row 4)
-        0 8 0 0 0 0 0 (Row 5)
-        8 8 0 0 0 0 0 (Row 6)
-    *   Step 1: Identify all 3-pixel L-shapes of color 8.
-        *   Shape 1: (0,5), (0,6), (1,6) - L-shape.
-            2x2 square: (0,5), (0,6), (1,5), (1,6).
-            Missing pixel: (1,5).
-        *   Shape 2: (1,0), (1,1), (2,0) - L-shape.
-            2x2 square: (1,0), (1,1), (2,0), (2,1).
-            Missing pixel: (2,1).
-        *   Shape 3: (3,3), (4,3), (4,4) - L-shape.
-            2x2 square: (3,3), (3,4), (4,3), (4,4).
-            Missing pixel: (3,4).
-        *   Shape 4: (5,1), (6,0), (6,1) - L-shape.
-            2x2 square: (5,0), (5,1), (6,0), (6,1).
-            Missing pixel: (5,0).
-    *   Step 2: Fill the missing pixels with color 1.
-        *   (1,5) = 1
-        *   (2,1) = 1
-        *   (3,4) = 1
-        *   (5,0) = 1
-    *   Test Input Grid:
+          <t xml:space="preserve">*   Input: 7x7 grid with 0s and 8s.
+    *   Rule: Identify 2x2 L-shapes (3 cells of 8s) and fill the missing 4th cell with 1.
+    *   Input Grid:
         Row 0: 0 0 0 0 0 8 8
         Row 1: 8 8 0 0 0 0 8
         Row 2: 8 0 0 0 0 0 0
@@ -521,12 +446,12 @@
         Row 4: 0 0 0 8 8 0 0
         Row 5: 0 8 0 0 0 0 0
         Row 6: 8 8 0 0 0 0 0
-    *   Applying changes:
-        (1,5) = 1: Row 1 becomes 8 8 0 0 0 1 8
-        (2,1) = 1: Row 2 becomes 8 1 0 0 0 0 0
-        (3,4) = 1: Row 3 becomes 0 0 0 8 1 0 0
-        (5,0) = 1: Row 5 becomes 1 8 0 0 0 0 0
-    *   Final Grid:
+    *   L-shapes and missing cells:
+        1.  (0,5), (0,6), (1,6) -&gt; Missing (1,5)
+        2.  (1,0), (1,1), (2,0) -&gt; Missing (2,1)
+        3.  (3,3), (4,3), (4,4) -&gt; Missing (3,4)
+        4.  (5,1), (6,0), (6,1) -&gt; Missing (5,0)
+    *   Final Grid Construction:
         Row 0: 0 0 0 0 0 8 8
         Row 1: 8 8 0 0 0 1 8
         Row 2: 8 1 0 0 0 0 0
@@ -534,66 +459,14 @@
         Row 4: 0 0 0 8 8 0 0
         Row 5: 1 8 0 0 0 0 0
         Row 6: 8 8 0 0 0 0 0
-    *   Example 1:
-        Input:
-        0 0 0 0 0 0 0
-        0 8 0 0 0 0 0
-        0 8 8 0 0 0 0
-        0 0 0 0 8 8 0
-        0 0 0 0 0 8 0
-        0 0 0 0 0 0 0
-        0 0 0 0 0 0 0
-        L-shape 1: (1,1), (2,1), (2,2). Missing: (1,2). (1,2) becomes 1. Correct.
-        L-shape 2: (3,4), (3,5), (4,5). Missing: (4,4). (4,4) becomes 1. Correct.
-    *   Example 2:
-        Input:
-        0 0 0 0 8 8 0
-        0 0 0 0 0 8 0
-        0 0 8 0 0 0 0
-        0 0 8 8 0 0 0
-        0 0 0 0 0 0 0
-        0 0 0 0 8 0 0
-        0 0 0 8 8 0 0
-        L-shape 1: (0,4), (0,5), (1,5). Missing: (1,4). (1,4) becomes 1. Correct.
-        L-shape 2: (2,2), (3,2), (3,3). Missing: (2,3). (2,3) becomes 1. Correct.
-        L-shape 3: (5,4), (6,3), (6,4). Missing: (5,3). (5,3) becomes 1. Correct.
-    *   Test Input:
-        0 0 0 0 0 8 8 (Row 0)
-        8 8 0 0 0 0 8 (Row 1)
-        8 0 0 0 0 0 0 (Row 2)
-        0 0 0 8 0 0 0 (Row 3)
-        0 0 0 8 8 0 0 (Row 4)
-        0 8 0 0 0 0 0 (Row 5)
-        8 8 0 0 0 0 0 (Row 6)
-        L-shapes of color 8:
-        1. (0,5), (0,6), (1,6) -&gt; Missing (1,5)
-        2. (1,0), (1,1), (2,0) -&gt; Missing (2,1)
-        3. (3,3), (4,3), (4,4) -&gt; Missing (3,4)
-        4. (5,1), (6,0), (6,1) -&gt; Missing (5,0)
-        Wait, let me double-check the coordinates for Shape 4.
-        (5,1) is Row 5, Col 1.
-        (6,0) is Row 6, Col 0.
-        (6,1) is Row 6, Col 1.
-        These three form an L-shape. The 2x2 square is (5,0), (5,1), (6,0), (6,1).
-        The missing pixel is (5,0). Correct.
-        Let me double-check Shape 1.
-        (0,5) is Row 0, Col 5.
-        (0,6) is Row 0, Col 6.
-        (1,6) is Row 1, Col 6.
-        These three form an L-shape. The 2x2 square is (0,5), (0,6), (1,5), (1,6).
-        The missing pixel is (1,5). Correct.
-        Let me double-check Shape 2.
-        (1,0) is Row 1, Col 0.
-        (1,1) is Row 1, Col 1.
-        (2,0) is Row 2, Col 0.
-        These three form an L-shape. The 2x2 square is (1,0), (1,1), (2,0), (2,1).
-        The missing pixel is (2,1). Correct.
-        Let me double-check Shape 3.
-        (3,3) is Row 3, Col 3.
-        (4,3) is Row 4, Col 3.
-        (4,4) is Row 4, Col 4.
-        These three form an L-shape. The 2x2 square is (3,3), (3,4), (4,3), (4,4).
-        The missing pixel is (3,4). Correct.</t>
+    *   Row 0: 0 0 0 0 0 8 8
+    *   Row 1: 8 8 0 0 0 1 8
+    *   Row 2: 8 1 0 0 0 0 0
+    *   Row 3: 0 0 0 8 1 0 0
+    *   Row 4: 0 0 0 8 8 0 0
+    *   Row 5: 1 8 0 0 0 0 0
+    *   Row 6: 8 8 0 0 0 0 0
+</t>
         </is>
       </c>
     </row>
@@ -605,147 +478,36 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">INCORRECT
-Reasoning:
-*   Input: A grid of size 12x12.
-    *   Colors: 0 (black/empty), 5 (grey).
-    *   Output: The same grid, but some 0s have been replaced by 2s (red).
-    *   Example 1:
-        *   Input has three grey shapes (color 5).
-        *   Shape 1: (2,1) to (5,4) - a 4x4 square with a hole. The hole is at (3,2), (3,3), (4,2), (4,3).
-        *   Shape 2: (4,7) to (7,10) - a 4x4 square with a hole. The hole is at (5,8), (6,8), (6,9).
-        *   Shape 3: (8,2) to (11,5) - a 4x4 square with a hole. The hole is at (10,3).
-        *   Output:
-            *   Shape 1's hole (3,2), (3,3), (4,2), (4,3) is filled with 2s.
-            *   Shape 2's hole (5,8), (6,8), (6,9) remains 0s.
-            *   Shape 3's hole (10,3) is filled with 2s.
-        *   *Wait, let me re-examine.*
-        *   Shape 1 hole: (3,2), (3,3), (4,2), (4,3). These are (row, col).
-            Input (3,2)=0, (3,3)=0, (4,2)=0, (4,3)=0.
-            Output (3,2)=2, (3,3)=2, (4,2)=2, (4,3)=2.
-        *   Shape 2 hole: (5,8), (6,8), (6,9).
-            Input (5,8)=0, (6,8)=0, (6,9)=0.
-            Output (5,8)=0, (6,8)=0, (6,9)=0.
-        *   Shape 3 hole: (10,3).
-            Input (10,3)=0.
-            Output (10,3)=2.
-    *   Example 2:
-        *   Shape 1: (1,1) to (4,4) - 4x4 square with a hole at (2,3).
-        *   Shape 2: (3,6) to (8,11) - 6x6 square with a hole from (4,7) to (7,10).
-        *   Shape 3: (7,0) to (11,4) - 5x5 square with a hole at (9,1), (9,2), (10,1), (10,2).
-        *   Output:
-            *   Shape 1 hole (2,3) filled with 2.
-            *   Shape 2 hole (4,7) to (7,10) filled with 2s.
-            *   Shape 3 hole (9,1), (9,2), (10,1), (10,2) filled with 2s.
-        *   *Wait, all holes are filled here? Let me re-check Example 1.*
-    *   Example 1 again:
-        *   Shape 1 hole: (3,2), (3,3), (4,2), (4,3) -&gt; filled with 2s.
-        *   Shape 2 hole: (5,8), (6,8), (6,9) -&gt; NOT filled.
-        *   Shape 3 hole: (10,3) -&gt; filled with 2s.
-        *   Wait, why was Shape 2's hole not filled?
-        *   Let's look at the shapes:
-            Shape 1: (2,1) to (5,4). Boundaries are all 5s. (It's a closed loop).
-            Shape 2: (4,7) to (7,10). Let's check the boundaries:
-                (4,7)=5, (4,8)=5, (4,9)=5, (4,10)=5
-                (5,7)=5, (5,8)=0, (5,9)=5, (5,10)=5
-                (6,7)=5, (6,8)=0, (6,9)=0, (6,10)=5
-                (7,7)=5, (7,8)=5, (7,9)=5, (7,10)=5
-                Wait, (5,8), (6,8), (6,9) are 0s. Is it a closed loop?
-                Yes, it's surrounded by 5s.
-                Wait, let me re-read Example 1 Output carefully.
-                Example 1 Output:
-                (3,2)=2, (3,3)=2, (4,2)=2, (4,3)=2 (Shape 1 hole)
-                (10,3)=2 (Shape 3 hole)
-                Shape 2 hole: (5,8)=0, (6,8)=0, (6,9)=0.
-                Wait, why is Shape 2's hole NOT filled? Let me re-examine Shape 2.
-                Input:
-                (4,7) 5 5 5 5 (4,10)
-                (5,7) 5 0 5 5 (5,10)
-                (6,7) 5 0 0 5 (6,10)
-                (7,7) 5 5 5 5 (7,10)
-                Looking at the input again:
-                Row 4: 0 5 0 0 5 0 0 5 5 5 5 0 (Col 7,8,9,10 are 5s)
-                Row 5: 0 5 5 5 5 0 0 5 0 5 5 0 (Col 7 is 5, Col 8 is 0, Col 9 is 5, Col 10 is 5)
-                Row 6: 0 0 0 0 0 0 0 5 0 0 5 0 (Col 7 is 5, Col 8 is 0, Col 9 is 0, Col 10 is 5)
-                Row 7: 0 0 0 0 0 0 0 5 5 5 5 0 (Col 7,8,9,10 are 5s)
-                Wait, (5,8) is 0, (6,8) is 0, (6,9) is 0.
-                Is it a closed loop?
-                (4,7) (4,8) (4,9) (4,10)
-                (5,7)  0    (5,9) (5,10)
-                (6,7)  0     0    (6,10)
-                (7,7) (7,8) (7,9) (7,10)
-                Yes, it is. Why is it not filled?
-    *   Wait, let me re-examine Example 3:
-        *   Shape 1: (1,1) to (6,5) - 6x5 square with hole from (2,2) to (5,4).
-        *   Shape 2: (3,7) to (6,10) - 4x4 square with hole from (4,8) to (5,9).
-        *   Shape 3: (8,3) to (11,8) - 4x6 square with hole from (9,4) to (10,7).
-        *   Output:
-            *   Shape 1 hole: (2,2) to (5,4) - NOT filled.
-            *   Shape 2 hole: (4,8) to (5,9) - filled with 2s.
-            *   Shape 3 hole: (9,4) to (10,7) - NOT filled.
-        *   *Wait, what's the pattern?*
-    *   Let's re-evaluate the holes that ARE filled:
-        Example 1:
-        - Shape 1 hole: (3,2), (3,3), (4,2), (4,3) - Filled.
-        - Shape 2 hole: (5,8), (6,8), (6,9) - Not filled.
-        - Shape 3 hole: (10,3) - Filled.
-        Example 2:
-        - Shape 1 hole: (2,3) - Filled.
-        - Shape 2 hole: (4,7) to (7,10) - Filled.
-        - Shape 3 hole: (9,1), (9,2), (10,1), (10,2) - Filled.
-        Example 3:
-        - Shape 1 hole: (2,2) to (5,4) - Not filled.
-        - Shape 2 hole: (4,8) to (5,9) - Filled.
-        - Shape 3 hole: (9,4) to (10,7) - Not filled.
-        Example 4:
-        - Shape 1 hole: (2,2), (2,3) - Not filled.
-        - Shape 2 hole: (7,4), (7,5), (8,4), (8,5), (9,4), (9,5), (9,6) - Not filled.
-    *   Wait, let me re-read Example 4 Output.
-        Example 4 Output is *identical* to Example 4 Input.
-        No 2s at all.
-        So in Example 4, none of the holes were filled.
-    *   Let's look at the holes again.
-        Example 1:
-        - Shape 1: hole is 2x2. (Filled)
-        - Shape 2: hole is 2x2 but one cell is filled? No, the hole is (5,8), (6,8), (6,9). That's 3 cells. (Not filled)
-        - Shape 3: hole is 1x1. (Filled)
-        Example 2:
-        - Shape 1: hole is 1x1. (Filled)
-        - Shape 2: hole is 4x4. (Filled)
-        - Shape 3: hole is 2x2. (Filled)
-        Example 3:
-        - Shape 1: hole is 4x3. (Not filled)
-        - Shape 2: hole is 2x2. (Filled)
-        - Shape 3: hole is 2x4. (Not filled)
-        Example 4:
-        - Shape 1: hole is 1x2. (Not filled)
-        - Shape 2: hole is 3x2 (approx). (Not filled)
-    *   Is there a pattern with the size of the hole?
-        Example 1: 2x2 (filled), 3 cells (not filled), 1x1 (filled).
-        Example 2: 1x1 (filled), 4x4 (filled), 2x2 (filled).
-        Example 3: 4x3 (not filled), 2x2 (filled), 2x4 (not filled).
-        Example 4: 1x2 (not filled), 3x2 (not filled).
-        Wait, in all the "filled" cases, the hole is a *square* (1x1, 2x2, 4x4).
-        Let's check:
-        Example 1:
-        Shape 1 hole: (3,2), (3,3), (4,2), (4,3) - 2x2 square. (Filled)
-        Shape 2 hole: (5,8), (6,8), (6,9) - Not a square. (Not filled)
-        Shape 3 hole: (10,3) - 1x1 square. (Filled)
-        Example 2:
-        Shape 1 hole: (2,3) - 1x1 square. (Filled)
-        Shape 2 hole: (4,7) to (7,10) - 4x4 square. (Filled)
-        Shape 3 hole: (9,1), (9,2), (10,1), (10,2) - 2x2 square. (Filled)
-        Example 3:
-        Shape 1 hole: (2,2) to (5,4) - 4x3 rectangle. (Not filled)
-        Shape 2 hole: (4,8) to (5,9) - 2x2 square. (Filled)
-        Shape 3 hole: (9,4) to (10,7) - 2x4 rectangle. (Not filled)
-        Example 4:
-        Shape 1 hole: (2,2), (2,3) - 1x2 rectangle. (Not filled)
-        Shape 2 hole: (7,4), (7,5), (8,4), (8,5), (9,4), (9,5), (9,6) - Not a square. (Not filled)
-        *Hypothesis: If a hole (a contiguous area of 0s surrounded by 5s) is a square, fill it with 2s.*
-    *   Let's test this hypothesis on the TEST INPUT.
-        TEST INPUT:
-        Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
+          <t xml:space="preserve">*   Input grid: 12x12.
+    *   Rule: If the interior 0s of a shape bounded by 5s form a square, fill them with 2s.
+    *   Shape 1: (1,0) to (5,4). Interior 0s: (2,1) to (4,3). This is a 3x3 square. Fill with 2s.
+    *   Shape 2: (1,7) to (5,10). Interior 0s: (2,9), (3,8), (3,9), (4,8), (4,9). Not a square.
+    *   Shape 3: (8,2) to (11,7). Interior 0s: (9,3) to (10,6). This is a 2x4 rectangle. Not a square.
+    *   Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
+    *   Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
+    *   Row 2: 5 2 2 2 5 0 0 5 5 0 5 0
+    *   Row 3: 5 2 2 2 5 0 0 5 0 0 5 0
+    *   Row 4: 5 2 2 2 5 0 0 5 0 0 5 0
+    *   Row 5: 5 5 5 5 5 0 0 5 5 5 5 0
+    *   Row 6: 0 0 0 0 0 0 0 0 0 0 0 0
+    *   Row 7: 0 0 0 0 0 0 0 0 0 0 0 0
+    *   Row 8: 0 0 5 5 5 5 5 5 0 0 0 0
+    *   Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
+    *   Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
+    *   Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
+    *   Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
+    *   Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
+    *   Row 2: 5 2 2 2 5 0 0 5 5 0 5 0
+    *   Row 3: 5 2 2 2 5 0 0 5 0 0 5 0
+    *   Row 4: 5 2 2 2 5 0 0 5 0 0 5 0
+    *   Row 5: 5 5 5 5 5 0 0 5 5 5 5 0
+    *   Row 6: 0 0 0 0 0 0 0 0 0 0 0 0
+    *   Row 7: 0 0 0 0 0 0 0 0 0 0 0 0
+    *   Row 8: 0 0 5 5 5 5 5 5 0 0 0 0
+    *   Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
+    *   Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
+    *   Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
+    *   Wait, let me re-check the input grid again.
         Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
         Row 2: 5 0 0 0 5 0 0 5 5 0 5 0
         Row 3: 5 0 0 0 5 0 0 5 0 0 5 0
@@ -757,32 +519,187 @@
         Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
         Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
         Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
-        Let's identify the holes:
         Shape 1: (1,0) to (5,4)
-        Hole 1: (2,1), (2,2), (2,3), (3,1), (3,2), (3,3), (4,1), (4,2), (4,3)
-        Size: 3x3. (It's a square!)
+        Row 1: 5 5 5 5 5
+        Row 2: 5 0 0 0 5
+        Row 3: 5 0 0 0 5
+        Row 4: 5 0 0 0 5
+        Row 5: 5 5 5 5 5
+        Interior: (2,1), (2,2), (2,3), (3,1), (3,2), (3,3), (4,1), (4,2), (4,3).
+        This is a 3x3 square. Correct.
         Shape 2: (1,7) to (5,10)
-        Hole 2: (2,9), (3,8), (3,9), (4,8), (4,9)
-        Wait, let me re-check Shape 2.
-        Row 1: (1,7)=5, (1,8)=5, (1,9)=5, (1,10)=5
-        Row 2: (2,7)=5, (2,8)=5, (2,9)=0, (2,10)=5
-        Row 3: (3,7)=5, (3,8)=0, (3,9)=0, (3,10)=5
-        Row 4: (4,7)=5, (4,8)=0, (4,9)=0, (4,10)=5
-        Row 5: (5,7)=5, (5,8)=5, (5,9)=5, (5,10)=5
-        Hole cells: (2,9), (3,8), (3,9), (4,8), (4,9).
-        This is not a square.
+        Row 1: 5 5 5 5
+        Row 2: 5 5 0 5
+        Row 3: 5 0 0 5
+        Row 4: 5 0 0 5
+        Row 5: 5 5 5 5
+        Interior: (2,9), (3,8), (3,9), (4,8), (4,9).
+        Not a square. Correct.
         Shape 3: (8,2) to (11,7)
-        Hole 3: (9,3), (9,4), (9,5), (9,6), (10,3), (10,4), (10,5), (10,6)
-        Size: 2x4. (Not a square).
-        So, only Hole 1 is a square (3x3).
-        Hole 1 cells:
-        (2,1), (2,2), (2,3)
-        (3,1), (3,2), (3,3)
-        (4,1), (4,2), (4,3)
-        These should be filled with 2s.
-    *   Let me double-check the other holes in the TEST INPUT one more time.
-        Shape 2:
-        Row 2, Col 9: </t>
+        Row 8: 5 5 5 5 5 5
+        Row 9: 5 0 0 0 0 5
+        Row 10: 5 0 0 0 0 5
+        Row 11: 5 5 5 5 5 5
+        Interior: (9,3), (9,4), (9,5), (9,6), (10,3), (10,4), (10,5), (10,6).
+        This is 2x4. Not a square. Correct.
+    *   Final check on the grid values:
+        Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
+        Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
+        Row 2: 5 2 2 2 5 0 0 5 5 0 5 0
+        Row 3: 5 2 2 2 5 0 0 5 0 0 5 0
+        Row 4: 5 2 2 2 5 0 0 5 0 0 5 0
+        Row 5: 5 5 5 5 5 0 0 5 5 5 5 0
+        Row 6: 0 0 0 0 0 0 0 0 0 0 0 0
+        Row 7: 0 0 0 0 0 0 0 0 0 0 0 0
+        Row 8: 0 0 5 5 5 5 5 5 0 0 0 0
+        Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
+        Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
+        Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>44f52bb0.json</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>The user wants me to extract the final predicted value from the provided reasoning text.
+The reasoning text analyzes several examples of 3x3 grids containing 0s and 2s and their corresponding 1x1 outputs (either 1 or 7).
+The reasoning concludes that if the grid is symmetric (horizontally or vertically), the output is 1; otherwise, it's 7.
+The test input provided in the reasoning text is:
+2 0 2
+2 2 2
+2 0 2
+The reasoning concludes that this grid is symmetric (both horizontally and vertically) and therefore the output should be 1.
+Final prediction: 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0a938d79.json</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>*   Grid size: 11 rows x 27 columns.
+    *   Points: (0, 5) = 3, (10, 10) = 4.
+    *   Δx = |5 - 10| = 5.
+    *   Δy = |0 - 10| = 10.
+    *   Δx &lt; Δy, so vertical stripes.
+    *   x_min = 5, color = 3.
+    *   x_max = 10, color = 4.
+    *   Columns: 5(3), 10(4), 15(3), 20(4), 25(3).
+    *   All other columns = 0.
+    *   All 11 rows are identical.
+    Row structure:
+    Col 0: 0
+    Col 1: 0
+    Col 2: 0
+    Col 3: 0
+    Col 4: 0
+    Col 5: 3
+    Col 6: 0
+    Col 7: 0
+    Col 8: 0
+    Col 9: 0
+    Col 10: 4
+    Col 11: 0
+    Col 12: 0
+    Col 13: 0
+    Col 14: 0
+    Col 15: 3
+    Col 16: 0
+    Col 17: 0
+    Col 18: 0
+    Col 19: 0
+    Col 20: 4
+    Col 21: 0
+    Col 22: 0
+    Col 23: 0
+    Col 24: 0
+    Col 25: 3
+    Col 26: 0
+    Row: `0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0`
+    Repeat this row 11 times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>00576224.json</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*   Input:
+        ```
+        3 2
+        7 8
+        ```
+    *   a = 3, b = 2, c = 7, d = 8
+    *   Row 1: a b a b a b -&gt; 3 2 3 2 3 2
+    *   Row 2: c d c d c d -&gt; 7 8 7 8 7 8
+    *   Row 3: b a b a b a -&gt; 2 3 2 3 2 3
+    *   Row 4: d c d c d c -&gt; 8 7 8 7 8 7
+    *   Row 5: a b a b a b -&gt; 3 2 3 2 3 2
+    *   Row 6: c d c d c d -&gt; 7 8 7 8 7 8
+    *   Row 1: 3 2 3 2 3 2
+    *   Row 2: 7 8 7 8 7 8
+    *   Row 3: 2 3 2 3 2 3
+    *   Row 4: 8 7 8 7 8 7
+    *   Row 5: 3 2 3 2 3 2
+    *   Row 6: 7 8 7 8 7 8
+    *   Is there any other pattern?
+        Example 1:
+        8 6 8 6 8 6
+        6 4 6 4 6 4
+        6 8 6 8 6 8
+        4 6 4 6 4 6
+        8 6 8 6 8 6
+        6 4 6 4 6 4
+        (a b a b a b)
+        (c d c d c d)
+        (b a b a b a)
+        (d c d c d c)
+        (a b a b a b)
+        (c d c d c d)
+        Yes, this is exactly what I've used.
+    *   Wait, let me re-read the Example 1 output one more time.
+        Example 1 Output:
+        8 6 8 6 8 6
+        6 4 6 4 6 4
+        6 8 6 8 6 8
+        4 6 4 6 4 6
+        8 6 8 6 8 6
+        6 4 6 4 6 4
+        Yes, it's exactly as I thought.
+    *   Let me re-read Example 2 output one more time.
+        Example 2 Output:
+        7 9 7 9 7 9
+        4 3 4 3 4 3
+        9 7 9 7 9 7
+        3 4 3 4 3 4
+        7 9 7 9 7 9
+        4 3 4 3 4 3
+        Yes, it's exactly as I thought.
+    *   Final check on the test input:
+        3 2
+        7 8
+        a=3, b=2, c=7, d=8
+        Row 1: 3 2 3 2 3 2
+        Row 2: 7 8 7 8 7 8
+        Row 3: 2 3 2 3 2 3
+        Row 4: 8 7 8 7 8 7
+        Row 5: 3 2 3 2 3 2
+        Row 6: 7 8 7 8 7 8
+</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adicionando progresso feito no lab
Novos testes foram feitos, com sucesso. Aqui estão algumas leves mudanças que eu fiz (no Tasks teste e no README) e resultados.
</commit_message>
<xml_diff>
--- a/batch_results.xlsx
+++ b/batch_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>gemma-4-31b-it</t>
         </is>
@@ -436,22 +448,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">*   Input: 7x7 grid with 0s and 8s.
-    *   Rule: Identify 2x2 L-shapes (3 cells of 8s) and fill the missing 4th cell with 1.
-    *   Input Grid:
-        Row 0: 0 0 0 0 0 8 8
-        Row 1: 8 8 0 0 0 0 8
-        Row 2: 8 0 0 0 0 0 0
-        Row 3: 0 0 0 8 0 0 0
-        Row 4: 0 0 0 8 8 0 0
-        Row 5: 0 8 0 0 0 0 0
-        Row 6: 8 8 0 0 0 0 0
-    *   L-shapes and missing cells:
-        1.  (0,5), (0,6), (1,6) -&gt; Missing (1,5)
-        2.  (1,0), (1,1), (2,0) -&gt; Missing (2,1)
-        3.  (3,3), (4,3), (4,4) -&gt; Missing (3,4)
-        4.  (5,1), (6,0), (6,1) -&gt; Missing (5,0)
-    *   Final Grid Construction:
+          <t>*   The goal is to extract the final predicted grid from the reasoning text.
+    *   The reasoning text describes a rule: find 2x2 areas where three cells are 8 and one is 0, and fill the 0 cell with 1.
+    *   The test input grid is:
+        0 0 0 0 0 8 8
+        8 8 0 0 0 0 8
+        8 0 0 0 0 0 0
+        0 0 0 8 0 0 0
+        0 0 0 8 8 0 0
+        0 8 0 0 0 0 0
+        8 8 0 0 0 0 0
+    *   The reasoning identifies the following 2x2 areas:
+        1.  (0,5), (0,6), (1,5), (1,6) -&gt; (1,5) becomes 1.
+        2.  (1,0), (1,1), (2,0), (2,1) -&gt; (2,1) becomes 1.
+        3.  (3,3), (3,4), (4,3), (4,4) -&gt; (3,4) becomes 1.
+        4.  (5,0), (5,1), (6,0), (6,1) -&gt; (5,0) becomes 1.
+    *   The final grid is constructed as:
         Row 0: 0 0 0 0 0 8 8
         Row 1: 8 8 0 0 0 1 8
         Row 2: 8 1 0 0 0 0 0
@@ -466,7 +478,72 @@
     *   Row 4: 0 0 0 8 8 0 0
     *   Row 5: 1 8 0 0 0 0 0
     *   Row 6: 8 8 0 0 0 0 0
-</t>
+    *   Wait, let me re-verify the coordinates one more time.
+        Input:
+        (0,5)=8, (0,6)=8
+        (1,0)=8, (1,1)=8, (1,6)=8
+        (2,0)=8
+        (3,3)=8
+        (4,3)=8, (4,4)=8
+        (5,1)=8
+        (6,0)=8, (6,1)=8
+        2x2s:
+        (0,5)(0,6)(1,5)(1,6): 8, 8, 0, 8 -&gt; (1,5)=1
+        (1,0)(1,1)(2,0)(2,1): 8, 8, 8, 0 -&gt; (2,1)=1
+        (3,3)(3,4)(4,3)(4,4): 8, 0, 8, 8 -&gt; (3,4)=1
+        (5,0)(5,1)(6,0)(6,1): 0, 8, 8, 8 -&gt; (5,0)=1
+        Final Grid:
+        0 0 0 0 0 8 8
+        8 8 0 0 0 1 8
+        8 1 0 0 0 0 0
+        0 0 0 8 1 0 0
+        0 0 0 8 8 0 0
+        1 8 0 0 0 0 0
+        8 8 0 0 0 0 0
+    *   Check the rows again:
+        Row 0: 0 0 0 0 0 8 8
+        Row 1: 8 8 0 0 0 1 8
+        Row 2: 8 1 0 0 0 0 0
+        Row 3: 0 0 0 8 1 0 0
+        Row 4: 0 0 0 8 8 0 0
+        Row 5: 1 8 0 0 0 0 0
+        Row 6: 8 8 0 0 0 0 0
+        (All rows have 7 elements).
+    *   Wait, let me re-read the input grid provided in the reasoning text:
+        0 0 0 0 0 8 8
+        8 8 0 0 0 0 8
+        8 0 0 0 0 0 0
+        0 0 0 8 0 0 0
+        0 0 0 8 8 0 0
+        0 8 0 0 0 0 0
+        8 8 0 0 0 0 0
+        (Yes, this matches).
+    *   Let me re-verify the 1s:
+        (1,5) - Row 1, Col 5. (0-indexed)
+        (2,1) - Row 2, Col 1.
+        (3,4) - Row 3, Col 4.
+        (5,0) - Row 5, Col 0.
+        Row 0: 0 0 0 0 0 8 8
+        Row 1: 8 8 0 0 0 1 8 (Col 5 is 1)
+        Row 2: 8 1 0 0 0 0 0 (Col 1 is 1)
+        Row 3: 0 0 0 8 1 0 0 (Col 4 is 1)
+        Row 4: 0 0 0 8 8 0 0
+        Row 5: 1 8 0 0 0 0 0 (Col 0 is 1)
+        Row 6: 8 8 0 0 0 0 0
+    *   Wait, let me re-check the 2x2 areas one more time.
+        (0,5)=8, (0,6)=8, (1,5)=0, (1,6)=8. (Three 8s, one 0). Correct.
+        (1,0)=8, (1,1)=8, (2,0)=8, (2,1)=0. (Three 8s, one 0). Correct.
+        (3,3)=8, (3,4)=0, (4,3)=8, (4,4)=8. (Three 8s, one 0). Correct.
+        (5,0)=0, (5,1)=8, (6,0)=8, (6,1)=8. (Three 8s, one 0). Correct.
+    *   Final check of the grid:
+        0 0 0 0 0 8 8
+        8 8 0 0 0 1 8
+        8 1 0 0 0 0 0
+        0 0 0 8 1 0 0
+        0 0 0 8 8 0 0
+        1 8 0 0 0 0 0
+        8 8 0 0 0 0 0
+        (7 rows, 7 columns).</t>
         </is>
       </c>
     </row>
@@ -478,71 +555,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">*   Input grid: 12x12.
-    *   Rule: If the interior 0s of a shape bounded by 5s form a square, fill them with 2s.
-    *   Shape 1: (1,0) to (5,4). Interior 0s: (2,1) to (4,3). This is a 3x3 square. Fill with 2s.
-    *   Shape 2: (1,7) to (5,10). Interior 0s: (2,9), (3,8), (3,9), (4,8), (4,9). Not a square.
-    *   Shape 3: (8,2) to (11,7). Interior 0s: (9,3) to (10,6). This is a 2x4 rectangle. Not a square.
-    *   Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
-    *   Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
-    *   Row 2: 5 2 2 2 5 0 0 5 5 0 5 0
-    *   Row 3: 5 2 2 2 5 0 0 5 0 0 5 0
-    *   Row 4: 5 2 2 2 5 0 0 5 0 0 5 0
-    *   Row 5: 5 5 5 5 5 0 0 5 5 5 5 0
-    *   Row 6: 0 0 0 0 0 0 0 0 0 0 0 0
-    *   Row 7: 0 0 0 0 0 0 0 0 0 0 0 0
-    *   Row 8: 0 0 5 5 5 5 5 5 0 0 0 0
-    *   Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
-    *   Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
-    *   Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
-    *   Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
-    *   Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
-    *   Row 2: 5 2 2 2 5 0 0 5 5 0 5 0
-    *   Row 3: 5 2 2 2 5 0 0 5 0 0 5 0
-    *   Row 4: 5 2 2 2 5 0 0 5 0 0 5 0
-    *   Row 5: 5 5 5 5 5 0 0 5 5 5 5 0
-    *   Row 6: 0 0 0 0 0 0 0 0 0 0 0 0
-    *   Row 7: 0 0 0 0 0 0 0 0 0 0 0 0
-    *   Row 8: 0 0 5 5 5 5 5 5 0 0 0 0
-    *   Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
-    *   Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
-    *   Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
-    *   Wait, let me re-check the input grid again.
-        Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
-        Row 2: 5 0 0 0 5 0 0 5 5 0 5 0
-        Row 3: 5 0 0 0 5 0 0 5 0 0 5 0
-        Row 4: 5 0 0 0 5 0 0 5 0 0 5 0
-        Row 5: 5 5 5 5 5 0 0 5 5 5 5 0
-        Row 6: 0 0 0 0 0 0 0 0 0 0 0 0
-        Row 7: 0 0 0 0 0 0 0 0 0 0 0 0
-        Row 8: 0 0 5 5 5 5 5 5 0 0 0 0
-        Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
-        Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
-        Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
-        Shape 1: (1,0) to (5,4)
-        Row 1: 5 5 5 5 5
-        Row 2: 5 0 0 0 5
-        Row 3: 5 0 0 0 5
-        Row 4: 5 0 0 0 5
-        Row 5: 5 5 5 5 5
-        Interior: (2,1), (2,2), (2,3), (3,1), (3,2), (3,3), (4,1), (4,2), (4,3).
-        This is a 3x3 square. Correct.
-        Shape 2: (1,7) to (5,10)
-        Row 1: 5 5 5 5
-        Row 2: 5 5 0 5
-        Row 3: 5 0 0 5
-        Row 4: 5 0 0 5
-        Row 5: 5 5 5 5
-        Interior: (2,9), (3,8), (3,9), (4,8), (4,9).
-        Not a square. Correct.
-        Shape 3: (8,2) to (11,7)
-        Row 8: 5 5 5 5 5 5
-        Row 9: 5 0 0 0 0 5
-        Row 10: 5 0 0 0 0 5
-        Row 11: 5 5 5 5 5 5
-        Interior: (9,3), (9,4), (9,5), (9,6), (10,3), (10,4), (10,5), (10,6).
-        This is 2x4. Not a square. Correct.
-    *   Final check on the grid values:
+          <t>The user wants me to extract the final predicted grid from the reasoning text.
+    *   Input grid:
+        0 0 0 0 0 0 0 0 0 0 0 0
+        5 5 5 5 5 0 0 5 5 5 5 0
+        5 0 0 0 5 0 0 5 5 0 5 0
+        5 0 0 0 5 0 0 5 0 0 5 0
+        5 0 0 0 5 0 0 5 0 0 5 0
+        5 5 5 5 5 0 0 5 5 5 5 0
+        0 0 0 0 0 0 0 0 0 0 0 0
+        0 0 0 0 0 0 0 0 0 0 0 0
+        0 0 5 5 5 5 5 5 0 0 0 0
+        0 0 5 0 0 0 0 5 0 0 0 0
+        0 0 5 0 0 0 0 5 0 0 0 0
+        0 0 5 5 5 5 5 5 0 0 0 0
+    *   Analysis from reasoning text:
+        *   Shape 1 (top-left): 3x3 square hole at (2,1) to (4,3). Fill with 2s.
+        *   Shape 2 (top-right): Non-square hole. Leave as 0s.
+        *   Shape 3 (bottom): 2x4 rectangle hole. Leave as 0s.
+    *   Applying the changes:
         Row 0: 0 0 0 0 0 0 0 0 0 0 0 0
         Row 1: 5 5 5 5 5 0 0 5 5 5 5 0
         Row 2: 5 2 2 2 5 0 0 5 5 0 5 0
@@ -555,7 +586,44 @@
         Row 9: 0 0 5 0 0 0 0 5 0 0 0 0
         Row 10: 0 0 5 0 0 0 0 5 0 0 0 0
         Row 11: 0 0 5 5 5 5 5 5 0 0 0 0
-</t>
+    *   Wait, let me re-verify the coordinates for Shape 1.
+        Input:
+        (1,0)=5 (1,1)=5 (1,2)=5 (1,3)=5 (1,4)=5
+        (2,0)=5 (2,1)=0 (2,2)=0 (2,3)=0 (2,4)=5
+        (3,0)=5 (3,1)=0 (3,2)=0 (3,3)=0 (3,4)=5
+        (4,0)=5 (4,1)=0 (4,2)=0 (4,3)=0 (4,4)=5
+        (5,0)=5 (5,1)=5 (5,2)=5 (5,3)=5 (5,4)=5
+        The hole is at (2,1), (2,2), (2,3), (3,1), (3,2), (3,3), (4,1), (4,2), (4,3).
+        These are rows 2, 3, 4 and columns 1, 2, 3.
+        Correct.
+    *   Let me re-verify Shape 2's hole.
+        (1,7)=5 (1,8)=5 (1,9)=5 (1,10)=5
+        (2,7)=5 (2,8)=5 (2,9)=0 (2,10)=5
+        (3,7)=5 (3,8)=0 (3,9)=0 (3,10)=5
+        (4,7)=5 (4,8)=0 (4,9)=0 (4,10)=5
+        (5,7)=5 (5,8)=5 (5,9)=5 (5,10)=5
+        Hole cells: (2,9), (3,8), (3,9), (4,8), (4,9).
+        These remain 0. Correct.
+    *   Let me re-verify Shape 3's hole.
+        (8,2)=5 (8,3)=5 (8,4)=5 (8,5)=5 (8,6)=5 (8,7)=5
+        (9,2)=5 (9,3)=0 (9,4)=0 (9,5)=0 (9,6)=0 (9,7)=5
+        (10,2)=5 (10,3)=0 (10,4)=0 (10,5)=0 (10,6)=0 (10,7)=5
+        (11,2)=5 (11,3)=5 (11,4)=5 (11,5)=5 (11,6)=5 (11,7)=5
+        Hole cells: (9,3), (9,4), (9,5), (9,6), (10,3), (10,4), (10,5), (10,6).
+        These remain 0. Correct.
+    *   Final Grid Construction:
+        0 0 0 0 0 0 0 0 0 0 0 0
+        5 5 5 5 5 0 0 5 5 5 5 0
+        5 2 2 2 5 0 0 5 5 0 5 0
+        5 2 2 2 5 0 0 5 0 0 5 0
+        5 2 2 2 5 0 0 5 0 0 5 0
+        5 5 5 5 5 0 0 5 5 5 5 0
+        0 0 0 0 0 0 0 0 0 0 0 0
+        0 0 0 0 0 0 0 0 0 0 0 0
+        0 0 5 5 5 5 5 5 0 0 0 0
+        0 0 5 0 0 0 0 5 0 0 0 0
+        0 0 5 0 0 0 0 5 0 0 0 0
+        0 0 5 5 5 5 5 5 0 0 0 0</t>
         </is>
       </c>
     </row>
@@ -568,14 +636,14 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>The user wants me to extract the final predicted value from the provided reasoning text.
-The reasoning text analyzes several examples of 3x3 grids containing 0s and 2s and their corresponding 1x1 outputs (either 1 or 7).
-The reasoning concludes that if the grid is symmetric (horizontally or vertically), the output is 1; otherwise, it's 7.
-The test input provided in the reasoning text is:
+The reasoning text analyzes several examples of 3x3 grids containing 0s and 2s, and their corresponding 1x1 outputs (either 1 or 7).
+The reasoning concludes that if the grid has reflectional symmetry (or an even number of corners with 2s), the output is 1.
+The test input is:
 2 0 2
 2 2 2
 2 0 2
-The reasoning concludes that this grid is symmetric (both horizontally and vertically) and therefore the output should be 1.
-Final prediction: 1.</t>
+This grid has both vertical and horizontal symmetry and 4 corners with 2s.
+The reasoning concludes the output should be 1.</t>
         </is>
       </c>
     </row>
@@ -587,119 +655,313 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>*   Grid size: 11 rows x 27 columns.
-    *   Points: (0, 5) = 3, (10, 10) = 4.
-    *   Δx = |5 - 10| = 5.
-    *   Δy = |0 - 10| = 10.
-    *   Δx &lt; Δy, so vertical stripes.
-    *   x_min = 5, color = 3.
-    *   x_max = 10, color = 4.
-    *   Columns: 5(3), 10(4), 15(3), 20(4), 25(3).
-    *   All other columns = 0.
-    *   All 11 rows are identical.
-    Row structure:
-    Col 0: 0
-    Col 1: 0
-    Col 2: 0
-    Col 3: 0
-    Col 4: 0
-    Col 5: 3
-    Col 6: 0
-    Col 7: 0
-    Col 8: 0
-    Col 9: 0
-    Col 10: 4
-    Col 11: 0
-    Col 12: 0
-    Col 13: 0
-    Col 14: 0
-    Col 15: 3
-    Col 16: 0
-    Col 17: 0
-    Col 18: 0
-    Col 19: 0
-    Col 20: 4
-    Col 21: 0
-    Col 22: 0
-    Col 23: 0
-    Col 24: 0
-    Col 25: 3
-    Col 26: 0
-    Row: `0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0`
-    Repeat this row 11 times.</t>
+          <t>*   Input: 11x27 grid.
+    *   P1: (0, 5) = 3
+    *   P2: (10, 10) = 4
+    *   Rule: r1=0, so use columns.
+    *   c1=5, c2=10.
+    *   Period = 2 * |10-5| = 10.
+    *   Columns for 3: 5, 15, 25.
+    *   Columns for 4: 10, 20.
+    *   Grid size: 11 rows, 27 columns.
+    *   All rows are identical.
+    *   Each row:
+        - Col 0-4: 0
+        - Col 5: 3
+        - Col 6-9: 0
+        - Col 10: 4
+        - Col 11-14: 0
+        - Col 15: 3
+        - Col 16-19: 0
+        - Col 20: 4
+        - Col 21-24: 0
+        - Col 25: 3
+        - Col 26: 0
+    *   Wait, let me double-check the column count.
+        0, 1, 2, 3, 4, 5(3), 6, 7, 8, 9, 10(4), 11, 12, 13, 14, 15(3), 16, 17, 18, 19, 20(4), 21, 22, 23, 24, 25(3), 26.
+        Total columns = 27. Correct.
+    *   Let's write out one row:
+        0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+        (Count: 5 zeros, 3, 4 zeros, 4, 4 zeros, 3, 4 zeros, 4, 4 zeros, 3, 1 zero)
+        5 + 1 + 4 + 1 + 4 + 1 + 4 + 1 + 4 + 1 + 1 = 27. Correct.
+    *   Now repeat this for 11 rows.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>0b148d64.json</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+    *   The reasoning text identifies four blocks of colors in the input grid.
+    *   The rule is to find the block with the unique color.
+    *   The blocks are:
+        *   Top-left: Color 1
+        *   Top-right: Color 3
+        *   Bottom-left: Color 3
+        *   Bottom-right: Color 3
+    *   The unique block is the top-left one.
+    *   The top-left block is:
+        Row 0: 1 1 1 1 0 1 0 0
+        Row 1: 1 0 1 0 1 1 0 0
+        Row 2: 1 1 0 1 1 0 0 0
+        Row 3: 0 0 0 1 1 1 0 0
+        Row 4: 1 1 1 1 1 1 0 0
+        Row 5: 1 1 1 1 1 1 0 0
+    *   The reasoning text states that all-zero columns should be excluded (based on Example 3).
+    *   Columns 6 and 7 are all zeros.
+    *   The resulting grid is:
+        1 1 1 1 0 1
+        1 0 1 0 1 1
+        1 1 0 1 1 0
+        0 0 0 1 1 1
+        1 1 1 1 1 1
+        1 1 1 1 1 1
+    Row 0: 1 1 1 1 0 1
+    Row 1: 1 0 1 0 1 1
+    Row 2: 1 1 0 1 1 0
+    Row 3: 0 0 0 1 1 1
+    Row 4: 1 1 1 1 1 1
+    Row 5: 1 1 1 1 1 1
+    Wait, let me re-read the reasoning text one more time to ensure I didn't miss any details.
+    "The resulting grid is 6x6:
+    Row 0: 1 1 1 1 0 1
+    Row 1: 1 0 1 0 1 1
+    Row 2: 1 1 0 1 1 0
+    Row 3: 0 0 0 1 1 1
+    Row 4: 1 1 1 1 1 1
+    Row 5: 1 1 1 1 1 1"
+    This matches my extraction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>00576224.json</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">*   Input:
-        ```
-        3 2
-        7 8
-        ```
-    *   a = 3, b = 2, c = 7, d = 8
-    *   Row 1: a b a b a b -&gt; 3 2 3 2 3 2
-    *   Row 2: c d c d c d -&gt; 7 8 7 8 7 8
-    *   Row 3: b a b a b a -&gt; 2 3 2 3 2 3
-    *   Row 4: d c d c d c -&gt; 8 7 8 7 8 7
-    *   Row 5: a b a b a b -&gt; 3 2 3 2 3 2
-    *   Row 6: c d c d c d -&gt; 7 8 7 8 7 8
-    *   Row 1: 3 2 3 2 3 2
-    *   Row 2: 7 8 7 8 7 8
-    *   Row 3: 2 3 2 3 2 3
-    *   Row 4: 8 7 8 7 8 7
-    *   Row 5: 3 2 3 2 3 2
-    *   Row 6: 7 8 7 8 7 8
-    *   Is there any other pattern?
-        Example 1:
-        8 6 8 6 8 6
-        6 4 6 4 6 4
-        6 8 6 8 6 8
-        4 6 4 6 4 6
-        8 6 8 6 8 6
-        6 4 6 4 6 4
-        (a b a b a b)
-        (c d c d c d)
-        (b a b a b a)
-        (d c d c d c)
-        (a b a b a b)
-        (c d c d c d)
-        Yes, this is exactly what I've used.
-    *   Wait, let me re-read the Example 1 output one more time.
-        Example 1 Output:
-        8 6 8 6 8 6
-        6 4 6 4 6 4
-        6 8 6 8 6 8
-        4 6 4 6 4 6
-        8 6 8 6 8 6
-        6 4 6 4 6 4
-        Yes, it's exactly as I thought.
-    *   Let me re-read Example 2 output one more time.
-        Example 2 Output:
-        7 9 7 9 7 9
-        4 3 4 3 4 3
-        9 7 9 7 9 7
-        3 4 3 4 3 4
-        7 9 7 9 7 9
-        4 3 4 3 4 3
-        Yes, it's exactly as I thought.
-    *   Final check on the test input:
-        3 2
-        7 8
-        a=3, b=2, c=7, d=8
-        Row 1: 3 2 3 2 3 2
-        Row 2: 7 8 7 8 7 8
-        Row 3: 2 3 2 3 2 3
-        Row 4: 8 7 8 7 8 7
-        Row 5: 3 2 3 2 3 2
-        Row 6: 7 8 7 8 7 8
-</t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>*   Input: 2x2 grid `[[3, 2], [7, 8]]`
+    *   Pattern:
+        *   Row 1: `a b a b a b` (3 2 3 2 3 2)
+        *   Row 2: `c d c d c d` (7 8 7 8 7 8)
+        *   Row 3: `b a b a b a` (2 3 2 3 2 3)
+        *   Row 4: `d c d c d c` (8 7 8 7 8 7)
+        *   Row 5: `a b a b a b` (3 2 3 2 3 2)
+        *   Row 6: `c d c d c d` (7 8 7 8 7 8)
+    *   Final Grid:
+        3 2 3 2 3 2
+        7 8 7 8 7 8
+        2 3 2 3 2 3
+        8 7 8 7 8 7
+        3 2 3 2 3 2
+        7 8 7 8 7 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0a1d4ef5.json</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+Looking at the reasoning text:
+- The user identified 4 rows of 3 blocks each.
+- Row 1: 2, 3, 3
+- Row 2: 4, 7, 1
+- Row 3: 1, 3, 7
+- Row 4: 4, 6, 2
+The final grid is:
+2 3 3
+4 7 1
+1 3 7
+4 6 2
+I must output only the &lt;prediction&gt; tags containing this grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0b17323b.json</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>*   Input: 15x15 grid with '1's at (0,0), (3,3), (6,6).
+    *   Pattern: Arithmetic progression with difference (3,3).
+    *   Next points: (9,9), (12,12).
+    *   Output: 15x15 grid with '1's at (0,0), (3,3), (6,6) and '2's at (9,9), (12,12).
+    Row 0: 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 1: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 2: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 3: 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0
+    Row 4: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 5: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 6: 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0
+    Row 7: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 8: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 9: 0 0 0 0 0 0 0 0 0 2 0 0 0 0 0
+    Row 10: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 11: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 12: 0 0 0 0 0 0 0 0 0 0 0 0 2 0 0
+    Row 13: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 14: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Wait, let me double-check the column indices.
+    (0,0) -&gt; Row 0, Col 0
+    (3,3) -&gt; Row 3, Col 3
+    (6,6) -&gt; Row 6, Col 6
+    (9,9) -&gt; Row 9, Col 9
+    (12,12) -&gt; Row 12, Col 12
+    Row 0: 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 1: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 2: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 3: 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0
+    Row 4: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 5: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 6: 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0
+    Row 7: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 8: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 9: 0 0 0 0 0 0 0 0 0 2 0 0 0 0 0
+    Row 10: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 11: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 12: 0 0 0 0 0 0 0 0 0 0 0 0 2 0 0
+    Row 13: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Row 14: 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+    Let's re-verify the column indices for Row 3, 6, 9, 12.
+    Row 3: Col 0, 1, 2, 3 (index 3)
+    Row 6: Col 0, 1, 2, 3, 4, 5, 6 (index 6)
+    Row 9: Col 0, 1, 2, 3, 4, 5, 6, 7, 8, 9 (index 9)
+    Row 12: Col 0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12 (index 12)
+    Yes, this is correct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0bb8deee.json</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+    *   TL (2s):
+        0 2 2
+        0 2 0
+        2 0 2
+    *   TR (3s):
+        3 3 3
+        0 3 3
+        3 0 0
+    *   BL (6s):
+        0 6 6
+        6 0 6
+        6 6 0
+    *   BR (4s):
+        0 4 0
+        4 0 4
+        0 4 0
+    *   Combine TL and TR (top half):
+        0 2 2 3 3 3
+        0 2 0 0 3 3
+        2 0 2 3 0 0
+    *   Combine BL and BR (bottom half):
+        0 6 6 0 4 0
+        6 0 6 4 0 4
+        6 6 0 0 4 0
+    0 2 2 3 3 3
+    0 2 0 0 3 3
+    2 0 2 3 0 0
+    0 6 6 0 4 0
+    6 0 6 4 0 4
+    6 6 0 0 4 0
+    *   TL:
+        Row 3: `0 0 2 2 0 0` (col 0-5) -&gt; col 1:0, 2:2, 3:2
+        Row 4: `0 0 2 0 0 0` (col 0-5) -&gt; col 1:0, 2:2, 3:0
+        Row 5: `0 2 0 2 0 0` (col 0-5) -&gt; col 1:2, 2:0, 3:2
+        (0 2 2 / 0 2 0 / 2 0 2) - Correct.
+    *   TR:
+        Row 2: `0 0 3 3 3 0` (col 7-12) -&gt; col 9:3, 10:3, 11:3
+        Row 3: `0 0 0 3 3 0` (col 7-12) -&gt; col 9:0, 10:3, 11:3
+        Row 4: `0 0 3 0 0 0` (col 7-12) -&gt; col 9:3, 10:0, 11:0
+        (3 3 3 / 0 3 3 / 3 0 0) - Correct.
+    *   BL:
+        Row 11: `0 0 6 6 0 0` (col 0-5) -&gt; col 1:0, 2:6, 3:6
+        Row 12: `0 6 0 6 0 0` (col 0-5) -&gt; col 1:6, 2:0, 3:6
+        Row 13: `0 6 6 0 0 0` (col 0-5) -&gt; col 1:6, 2:6, 3:0
+        (0 6 6 / 6 0 6 / 6 6 0) - Correct.
+    *   BR:
+        Row 10: `0 0 0 4 0 0` (col 7-12) -&gt; col 9:0, 10:4, 11:0
+        Row 11: `0 0 4 0 4 0` (col 7-12) -&gt; col 9:4, 10:0, 11:4
+        Row 12: `0 0 0 4 0 0` (col 7-12) -&gt; col 9:0, 10:4, 11:0
+        (0 4 0 / 4 0 4 / 0 4 0) - Correct.
+    0 2 2 3 3 3
+    0 2 0 0 3 3
+    2 0 2 3 0 0
+    0 6 6 0 4 0
+    6 0 6 4 0 4
+    6 6 0 0 4 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0becf7df.json</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+    *   The reasoning text describes a pattern where a 2x2 block at the top-left (0,0 to 1,1) defines a color mapping.
+    *   Mapping: (0,0) &lt;-&gt; (0,1) and (1,0) &lt;-&gt; (1,1).
+    *   For the test input:
+        (0,0)=8, (0,1)=9 =&gt; 8 &lt;-&gt; 9
+        (1,0)=2, (1,1)=4 =&gt; 2 &lt;-&gt; 4
+    *   The 2x2 block itself remains unchanged.
+    *   All other cells in the grid are updated based on this mapping.
+    *   Input Grid:
+        Row 0: 8 9 0 0 0 0 0 0 0 0
+        Row 1: 2 4 0 0 0 9 9 0 0 0
+        Row 2: 0 0 0 8 8 8 9 0 0 0
+        Row 3: 0 0 0 2 8 8 9 0 0 0
+        Row 4: 0 0 0 2 4 2 0 0 0 0
+        Row 5: 0 0 0 2 2 4 0 0 0 0
+        Row 6: 0 0 0 2 4 4 0 0 0 0
+        Row 7: 0 0 0 9 4 4 0 0 0 0
+        Row 8: 0 0 0 0 0 4 0 0 0 0
+        Row 9: 0 0 0 0 0 0 0 0 0 0
+    *   Applying Mapping (8&lt;-&gt;9, 2&lt;-&gt;4):
+        Row 0: 8 9 0 0 0 0 0 0 0 0 (Unchanged)
+        Row 1: 2 4 0 0 0 8 8 0 0 0 (9-&gt;8)
+        Row 2: 0 0 0 9 9 9 8 0 0 0 (8-&gt;9, 9-&gt;8)
+        Row 3: 0 0 0 4 9 9 8 0 0 0 (2-&gt;4, 8-&gt;9, 9-&gt;8)
+        Row 4: 0 0 0 4 2 4 0 0 0 0 (2-&gt;4, 4-&gt;2, 2-&gt;4)
+        Row 5: 0 0 0 4 4 2 0 0 0 0 (2-&gt;4, 2-&gt;4, 4-&gt;2)
+        Row 6: 0 0 0 4 2 2 0 0 0 0 (2-&gt;4, 4-&gt;2, 4-&gt;2)
+        Row 7: 0 0 0 8 2 2 0 0 0 0 (9-&gt;8, 4-&gt;2, 4-&gt;2)
+        Row 8: 0 0 0 0 0 2 0 0 0 0 (4-&gt;2)
+        Row 9: 0 0 0 0 0 0 0 0 0 0 (Unchanged)
+    Row 0: 8 9 0 0 0 0 0 0 0 0
+    Row 1: 2 4 0 0 0 8 8 0 0 0
+    Row 2: 0 0 0 9 9 9 8 0 0 0
+    Row 3: 0 0 0 4 9 9 8 0 0 0
+    Row 4: 0 0 0 4 2 4 0 0 0 0
+    Row 5: 0 0 0 4 4 2 0 0 0 0
+    Row 6: 0 0 0 4 2 2 0 0 0 0
+    Row 7: 0 0 0 8 2 2 0 0 0 0
+    Row 8: 0 0 0 0 0 2 0 0 0 0
+    Row 9: 0 0 0 0 0 0 0 0 0 0</t>
         </is>
       </c>
     </row>

</xml_diff>